<commit_message>
Actualiza histórico prdemcad + csv
</commit_message>
<xml_diff>
--- a/Historico_prdemcad.xlsx
+++ b/Historico_prdemcad.xlsx
@@ -30292,7 +30292,7 @@
         <v>3</v>
       </c>
       <c r="G1106" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1107">
@@ -30319,7 +30319,7 @@
         <v>3</v>
       </c>
       <c r="G1107" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1108">
@@ -30346,7 +30346,7 @@
         <v>3</v>
       </c>
       <c r="G1108" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1109">
@@ -30373,7 +30373,7 @@
         <v>3</v>
       </c>
       <c r="G1109" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1110">
@@ -30400,7 +30400,7 @@
         <v>3</v>
       </c>
       <c r="G1110" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1111">
@@ -30427,7 +30427,7 @@
         <v>3</v>
       </c>
       <c r="G1111" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1112">
@@ -30454,7 +30454,7 @@
         <v>3</v>
       </c>
       <c r="G1112" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1113">
@@ -30481,7 +30481,7 @@
         <v>3</v>
       </c>
       <c r="G1113" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1114">
@@ -30508,7 +30508,7 @@
         <v>3</v>
       </c>
       <c r="G1114" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1115">
@@ -30535,7 +30535,7 @@
         <v>3</v>
       </c>
       <c r="G1115" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1116">
@@ -30562,7 +30562,7 @@
         <v>3</v>
       </c>
       <c r="G1116" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1117">
@@ -30589,7 +30589,7 @@
         <v>3</v>
       </c>
       <c r="G1117" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1118">
@@ -30616,7 +30616,7 @@
         <v>3</v>
       </c>
       <c r="G1118" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1119">
@@ -30643,7 +30643,7 @@
         <v>3</v>
       </c>
       <c r="G1119" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1120">
@@ -30670,7 +30670,7 @@
         <v>3</v>
       </c>
       <c r="G1120" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1121">
@@ -30697,7 +30697,7 @@
         <v>3</v>
       </c>
       <c r="G1121" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1122">
@@ -30724,7 +30724,7 @@
         <v>3</v>
       </c>
       <c r="G1122" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1123">
@@ -30751,7 +30751,7 @@
         <v>3</v>
       </c>
       <c r="G1123" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1124">
@@ -30778,7 +30778,7 @@
         <v>3</v>
       </c>
       <c r="G1124" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1125">
@@ -30805,7 +30805,7 @@
         <v>3</v>
       </c>
       <c r="G1125" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1126">
@@ -30832,7 +30832,7 @@
         <v>3</v>
       </c>
       <c r="G1126" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1127">
@@ -30859,7 +30859,7 @@
         <v>3</v>
       </c>
       <c r="G1127" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1128">
@@ -30886,7 +30886,7 @@
         <v>3</v>
       </c>
       <c r="G1128" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1129">
@@ -30913,7 +30913,7 @@
         <v>3</v>
       </c>
       <c r="G1129" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1130">
@@ -30940,7 +30940,7 @@
         <v>3</v>
       </c>
       <c r="G1130" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1131">
@@ -30967,7 +30967,7 @@
         <v>3</v>
       </c>
       <c r="G1131" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1132">
@@ -30994,7 +30994,7 @@
         <v>3</v>
       </c>
       <c r="G1132" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1133">
@@ -31021,7 +31021,7 @@
         <v>3</v>
       </c>
       <c r="G1133" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1134">
@@ -31048,7 +31048,7 @@
         <v>3</v>
       </c>
       <c r="G1134" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1135">
@@ -31075,7 +31075,7 @@
         <v>3</v>
       </c>
       <c r="G1135" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1136">
@@ -31102,7 +31102,7 @@
         <v>3</v>
       </c>
       <c r="G1136" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1137">
@@ -31129,7 +31129,7 @@
         <v>3</v>
       </c>
       <c r="G1137" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1138">
@@ -31156,7 +31156,7 @@
         <v>3</v>
       </c>
       <c r="G1138" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1139">
@@ -31183,7 +31183,7 @@
         <v>3</v>
       </c>
       <c r="G1139" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1140">
@@ -31210,7 +31210,7 @@
         <v>3</v>
       </c>
       <c r="G1140" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1141">
@@ -31237,7 +31237,7 @@
         <v>3</v>
       </c>
       <c r="G1141" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1142">
@@ -31264,7 +31264,7 @@
         <v>3</v>
       </c>
       <c r="G1142" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1143">
@@ -31291,7 +31291,7 @@
         <v>3</v>
       </c>
       <c r="G1143" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1144">
@@ -31318,7 +31318,7 @@
         <v>3</v>
       </c>
       <c r="G1144" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1145">
@@ -31345,7 +31345,7 @@
         <v>3</v>
       </c>
       <c r="G1145" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1146">
@@ -31372,7 +31372,7 @@
         <v>3</v>
       </c>
       <c r="G1146" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1147">
@@ -31399,7 +31399,7 @@
         <v>3</v>
       </c>
       <c r="G1147" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1148">
@@ -31426,7 +31426,7 @@
         <v>3</v>
       </c>
       <c r="G1148" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1149">
@@ -31453,7 +31453,7 @@
         <v>3</v>
       </c>
       <c r="G1149" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1150">
@@ -31480,7 +31480,7 @@
         <v>3</v>
       </c>
       <c r="G1150" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1151">
@@ -31507,7 +31507,7 @@
         <v>3</v>
       </c>
       <c r="G1151" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1152">
@@ -31534,7 +31534,7 @@
         <v>3</v>
       </c>
       <c r="G1152" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1153">
@@ -31561,7 +31561,7 @@
         <v>3</v>
       </c>
       <c r="G1153" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1154">
@@ -31588,7 +31588,7 @@
         <v>3</v>
       </c>
       <c r="G1154" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1155">
@@ -31615,7 +31615,7 @@
         <v>3</v>
       </c>
       <c r="G1155" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1156">
@@ -31642,7 +31642,7 @@
         <v>3</v>
       </c>
       <c r="G1156" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1157">
@@ -31669,7 +31669,7 @@
         <v>3</v>
       </c>
       <c r="G1157" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1158">
@@ -31696,7 +31696,7 @@
         <v>3</v>
       </c>
       <c r="G1158" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1159">
@@ -31723,7 +31723,7 @@
         <v>3</v>
       </c>
       <c r="G1159" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1160">
@@ -31750,7 +31750,7 @@
         <v>3</v>
       </c>
       <c r="G1160" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1161">
@@ -31777,7 +31777,7 @@
         <v>3</v>
       </c>
       <c r="G1161" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1162">
@@ -31804,7 +31804,7 @@
         <v>3</v>
       </c>
       <c r="G1162" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1163">
@@ -31831,7 +31831,7 @@
         <v>3</v>
       </c>
       <c r="G1163" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1164">
@@ -31858,7 +31858,7 @@
         <v>3</v>
       </c>
       <c r="G1164" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1165">
@@ -31885,7 +31885,7 @@
         <v>3</v>
       </c>
       <c r="G1165" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1166">
@@ -31912,7 +31912,7 @@
         <v>3</v>
       </c>
       <c r="G1166" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1167">
@@ -31939,7 +31939,7 @@
         <v>3</v>
       </c>
       <c r="G1167" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1168">
@@ -31966,7 +31966,7 @@
         <v>3</v>
       </c>
       <c r="G1168" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1169">
@@ -31993,7 +31993,7 @@
         <v>3</v>
       </c>
       <c r="G1169" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1170">
@@ -32020,7 +32020,7 @@
         <v>3</v>
       </c>
       <c r="G1170" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1171">
@@ -32047,7 +32047,7 @@
         <v>3</v>
       </c>
       <c r="G1171" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1172">
@@ -32074,7 +32074,7 @@
         <v>3</v>
       </c>
       <c r="G1172" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1173">
@@ -32101,7 +32101,7 @@
         <v>3</v>
       </c>
       <c r="G1173" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1174">
@@ -32128,7 +32128,7 @@
         <v>3</v>
       </c>
       <c r="G1174" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1175">
@@ -32155,7 +32155,7 @@
         <v>3</v>
       </c>
       <c r="G1175" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1176">
@@ -32182,7 +32182,7 @@
         <v>3</v>
       </c>
       <c r="G1176" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1177">
@@ -32209,7 +32209,7 @@
         <v>3</v>
       </c>
       <c r="G1177" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1178">
@@ -32236,7 +32236,7 @@
         <v>3</v>
       </c>
       <c r="G1178" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1179">
@@ -32263,7 +32263,7 @@
         <v>3</v>
       </c>
       <c r="G1179" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1180">
@@ -32290,7 +32290,7 @@
         <v>3</v>
       </c>
       <c r="G1180" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1181">
@@ -32317,7 +32317,7 @@
         <v>3</v>
       </c>
       <c r="G1181" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1182">
@@ -32344,7 +32344,7 @@
         <v>3</v>
       </c>
       <c r="G1182" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1183">
@@ -32371,7 +32371,7 @@
         <v>3</v>
       </c>
       <c r="G1183" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1184">
@@ -32398,7 +32398,7 @@
         <v>3</v>
       </c>
       <c r="G1184" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1185">
@@ -32425,7 +32425,7 @@
         <v>3</v>
       </c>
       <c r="G1185" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1186">
@@ -32452,7 +32452,7 @@
         <v>3</v>
       </c>
       <c r="G1186" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1187">
@@ -32479,7 +32479,7 @@
         <v>3</v>
       </c>
       <c r="G1187" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1188">
@@ -32506,7 +32506,7 @@
         <v>3</v>
       </c>
       <c r="G1188" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1189">
@@ -32533,7 +32533,7 @@
         <v>3</v>
       </c>
       <c r="G1189" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1190">
@@ -32560,7 +32560,7 @@
         <v>3</v>
       </c>
       <c r="G1190" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1191">
@@ -32587,7 +32587,7 @@
         <v>3</v>
       </c>
       <c r="G1191" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1192">
@@ -32614,7 +32614,7 @@
         <v>3</v>
       </c>
       <c r="G1192" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1193">
@@ -32641,7 +32641,7 @@
         <v>3</v>
       </c>
       <c r="G1193" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1194">
@@ -32668,7 +32668,7 @@
         <v>3</v>
       </c>
       <c r="G1194" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1195">
@@ -32695,7 +32695,7 @@
         <v>3</v>
       </c>
       <c r="G1195" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1196">
@@ -32722,7 +32722,7 @@
         <v>3</v>
       </c>
       <c r="G1196" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1197">
@@ -32749,7 +32749,7 @@
         <v>3</v>
       </c>
       <c r="G1197" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1198">
@@ -32776,7 +32776,7 @@
         <v>3</v>
       </c>
       <c r="G1198" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1199">
@@ -32803,7 +32803,7 @@
         <v>3</v>
       </c>
       <c r="G1199" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1200">
@@ -32830,7 +32830,7 @@
         <v>3</v>
       </c>
       <c r="G1200" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1201">
@@ -32857,7 +32857,7 @@
         <v>3</v>
       </c>
       <c r="G1201" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1202">
@@ -32884,7 +32884,7 @@
         <v>3</v>
       </c>
       <c r="G1202" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1203">
@@ -32911,7 +32911,7 @@
         <v>3</v>
       </c>
       <c r="G1203" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1204">
@@ -32938,7 +32938,7 @@
         <v>3</v>
       </c>
       <c r="G1204" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1205">
@@ -32965,7 +32965,7 @@
         <v>3</v>
       </c>
       <c r="G1205" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1206">
@@ -32992,7 +32992,7 @@
         <v>3</v>
       </c>
       <c r="G1206" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1207">
@@ -33019,7 +33019,7 @@
         <v>3</v>
       </c>
       <c r="G1207" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1208">
@@ -33046,7 +33046,7 @@
         <v>3</v>
       </c>
       <c r="G1208" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1209">
@@ -33073,7 +33073,7 @@
         <v>3</v>
       </c>
       <c r="G1209" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1210">
@@ -33100,7 +33100,7 @@
         <v>3</v>
       </c>
       <c r="G1210" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1211">
@@ -33127,7 +33127,7 @@
         <v>3</v>
       </c>
       <c r="G1211" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1212">
@@ -33154,7 +33154,7 @@
         <v>3</v>
       </c>
       <c r="G1212" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1213">
@@ -33181,7 +33181,7 @@
         <v>3</v>
       </c>
       <c r="G1213" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1214">
@@ -33208,7 +33208,7 @@
         <v>3</v>
       </c>
       <c r="G1214" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1215">
@@ -33235,7 +33235,7 @@
         <v>3</v>
       </c>
       <c r="G1215" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1216">
@@ -33262,7 +33262,7 @@
         <v>3</v>
       </c>
       <c r="G1216" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1217">
@@ -33289,7 +33289,7 @@
         <v>3</v>
       </c>
       <c r="G1217" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1218">
@@ -33316,7 +33316,7 @@
         <v>3</v>
       </c>
       <c r="G1218" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1219">
@@ -33343,7 +33343,7 @@
         <v>3</v>
       </c>
       <c r="G1219" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1220">
@@ -33370,7 +33370,7 @@
         <v>3</v>
       </c>
       <c r="G1220" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1221">
@@ -33397,7 +33397,7 @@
         <v>3</v>
       </c>
       <c r="G1221" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1222">
@@ -33424,7 +33424,7 @@
         <v>3</v>
       </c>
       <c r="G1222" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1223">
@@ -33451,7 +33451,7 @@
         <v>3</v>
       </c>
       <c r="G1223" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1224">
@@ -33478,7 +33478,7 @@
         <v>3</v>
       </c>
       <c r="G1224" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1225">
@@ -33505,7 +33505,7 @@
         <v>3</v>
       </c>
       <c r="G1225" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1226">
@@ -33532,7 +33532,7 @@
         <v>3</v>
       </c>
       <c r="G1226" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1227">
@@ -33559,7 +33559,7 @@
         <v>3</v>
       </c>
       <c r="G1227" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1228">
@@ -33586,7 +33586,7 @@
         <v>3</v>
       </c>
       <c r="G1228" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1229">
@@ -33613,7 +33613,7 @@
         <v>3</v>
       </c>
       <c r="G1229" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1230">
@@ -33640,7 +33640,7 @@
         <v>3</v>
       </c>
       <c r="G1230" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1231">
@@ -33667,7 +33667,7 @@
         <v>3</v>
       </c>
       <c r="G1231" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1232">
@@ -33694,7 +33694,7 @@
         <v>3</v>
       </c>
       <c r="G1232" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1233">
@@ -33721,7 +33721,7 @@
         <v>3</v>
       </c>
       <c r="G1233" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1234">
@@ -33748,7 +33748,7 @@
         <v>3</v>
       </c>
       <c r="G1234" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1235">
@@ -33775,7 +33775,7 @@
         <v>3</v>
       </c>
       <c r="G1235" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1236">
@@ -33802,7 +33802,7 @@
         <v>3</v>
       </c>
       <c r="G1236" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1237">
@@ -33829,7 +33829,7 @@
         <v>3</v>
       </c>
       <c r="G1237" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1238">
@@ -33856,7 +33856,7 @@
         <v>3</v>
       </c>
       <c r="G1238" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1239">
@@ -33883,7 +33883,7 @@
         <v>3</v>
       </c>
       <c r="G1239" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1240">
@@ -33910,7 +33910,7 @@
         <v>3</v>
       </c>
       <c r="G1240" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1241">
@@ -33937,7 +33937,7 @@
         <v>3</v>
       </c>
       <c r="G1241" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1242">
@@ -33964,7 +33964,7 @@
         <v>3</v>
       </c>
       <c r="G1242" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1243">
@@ -33991,7 +33991,7 @@
         <v>3</v>
       </c>
       <c r="G1243" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1244">
@@ -34018,7 +34018,7 @@
         <v>3</v>
       </c>
       <c r="G1244" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1245">
@@ -34045,7 +34045,7 @@
         <v>3</v>
       </c>
       <c r="G1245" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1246">
@@ -34072,7 +34072,7 @@
         <v>3</v>
       </c>
       <c r="G1246" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1247">
@@ -34099,7 +34099,7 @@
         <v>3</v>
       </c>
       <c r="G1247" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1248">
@@ -34126,7 +34126,7 @@
         <v>3</v>
       </c>
       <c r="G1248" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1249">
@@ -34153,7 +34153,7 @@
         <v>3</v>
       </c>
       <c r="G1249" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1250">
@@ -34180,7 +34180,7 @@
         <v>3</v>
       </c>
       <c r="G1250" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1251">
@@ -34207,7 +34207,7 @@
         <v>3</v>
       </c>
       <c r="G1251" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1252">
@@ -34234,7 +34234,7 @@
         <v>3</v>
       </c>
       <c r="G1252" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1253">
@@ -34261,7 +34261,7 @@
         <v>3</v>
       </c>
       <c r="G1253" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1254">
@@ -34288,7 +34288,7 @@
         <v>3</v>
       </c>
       <c r="G1254" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1255">
@@ -34315,7 +34315,7 @@
         <v>3</v>
       </c>
       <c r="G1255" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1256">
@@ -34342,7 +34342,7 @@
         <v>3</v>
       </c>
       <c r="G1256" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1257">
@@ -34369,7 +34369,7 @@
         <v>3</v>
       </c>
       <c r="G1257" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1258">
@@ -34396,7 +34396,7 @@
         <v>3</v>
       </c>
       <c r="G1258" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1259">
@@ -34423,7 +34423,7 @@
         <v>3</v>
       </c>
       <c r="G1259" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1260">
@@ -34450,7 +34450,7 @@
         <v>3</v>
       </c>
       <c r="G1260" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1261">
@@ -34477,7 +34477,7 @@
         <v>3</v>
       </c>
       <c r="G1261" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1262">
@@ -34504,7 +34504,7 @@
         <v>3</v>
       </c>
       <c r="G1262" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1263">
@@ -34531,7 +34531,7 @@
         <v>3</v>
       </c>
       <c r="G1263" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1264">
@@ -34558,7 +34558,7 @@
         <v>3</v>
       </c>
       <c r="G1264" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1265">
@@ -34585,7 +34585,7 @@
         <v>3</v>
       </c>
       <c r="G1265" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1266">
@@ -34612,7 +34612,7 @@
         <v>3</v>
       </c>
       <c r="G1266" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1267">
@@ -34639,7 +34639,7 @@
         <v>3</v>
       </c>
       <c r="G1267" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1268">
@@ -34666,7 +34666,7 @@
         <v>3</v>
       </c>
       <c r="G1268" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1269">
@@ -34693,7 +34693,7 @@
         <v>3</v>
       </c>
       <c r="G1269" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1270">
@@ -34720,7 +34720,7 @@
         <v>3</v>
       </c>
       <c r="G1270" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1271">
@@ -34747,7 +34747,7 @@
         <v>3</v>
       </c>
       <c r="G1271" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1272">
@@ -34774,7 +34774,7 @@
         <v>3</v>
       </c>
       <c r="G1272" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1273">
@@ -34801,7 +34801,7 @@
         <v>3</v>
       </c>
       <c r="G1273" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1274">
@@ -34828,7 +34828,7 @@
         <v>3</v>
       </c>
       <c r="G1274" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1275">
@@ -34855,7 +34855,7 @@
         <v>3</v>
       </c>
       <c r="G1275" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1276">
@@ -34882,7 +34882,7 @@
         <v>3</v>
       </c>
       <c r="G1276" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1277">
@@ -34909,7 +34909,7 @@
         <v>3</v>
       </c>
       <c r="G1277" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1278">
@@ -34936,7 +34936,7 @@
         <v>3</v>
       </c>
       <c r="G1278" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1279">
@@ -34963,7 +34963,7 @@
         <v>3</v>
       </c>
       <c r="G1279" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1280">
@@ -34990,7 +34990,7 @@
         <v>3</v>
       </c>
       <c r="G1280" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1281">
@@ -35017,7 +35017,7 @@
         <v>3</v>
       </c>
       <c r="G1281" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1282">
@@ -35044,7 +35044,7 @@
         <v>3</v>
       </c>
       <c r="G1282" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1283">
@@ -35071,7 +35071,7 @@
         <v>3</v>
       </c>
       <c r="G1283" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1284">
@@ -35098,7 +35098,7 @@
         <v>3</v>
       </c>
       <c r="G1284" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1285">
@@ -35125,7 +35125,7 @@
         <v>3</v>
       </c>
       <c r="G1285" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1286">
@@ -35152,7 +35152,7 @@
         <v>3</v>
       </c>
       <c r="G1286" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1287">
@@ -35179,7 +35179,7 @@
         <v>3</v>
       </c>
       <c r="G1287" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1288">
@@ -35206,7 +35206,7 @@
         <v>3</v>
       </c>
       <c r="G1288" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1289">
@@ -35233,7 +35233,7 @@
         <v>3</v>
       </c>
       <c r="G1289" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1290">
@@ -35260,7 +35260,7 @@
         <v>3</v>
       </c>
       <c r="G1290" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1291">
@@ -35287,7 +35287,7 @@
         <v>3</v>
       </c>
       <c r="G1291" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1292">
@@ -35314,7 +35314,7 @@
         <v>3</v>
       </c>
       <c r="G1292" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1293">
@@ -35341,7 +35341,7 @@
         <v>3</v>
       </c>
       <c r="G1293" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1294">
@@ -35368,7 +35368,7 @@
         <v>3</v>
       </c>
       <c r="G1294" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1295">
@@ -35395,7 +35395,7 @@
         <v>3</v>
       </c>
       <c r="G1295" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1296">
@@ -35422,7 +35422,7 @@
         <v>3</v>
       </c>
       <c r="G1296" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1297">
@@ -35449,7 +35449,7 @@
         <v>3</v>
       </c>
       <c r="G1297" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1298">
@@ -35476,7 +35476,7 @@
         <v>3</v>
       </c>
       <c r="G1298" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1299">
@@ -35503,7 +35503,7 @@
         <v>3</v>
       </c>
       <c r="G1299" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1300">
@@ -35530,7 +35530,7 @@
         <v>3</v>
       </c>
       <c r="G1300" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1301">
@@ -35557,7 +35557,7 @@
         <v>3</v>
       </c>
       <c r="G1301" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1302">
@@ -35584,7 +35584,7 @@
         <v>3</v>
       </c>
       <c r="G1302" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1303">
@@ -35611,7 +35611,7 @@
         <v>3</v>
       </c>
       <c r="G1303" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1304">
@@ -35638,7 +35638,7 @@
         <v>3</v>
       </c>
       <c r="G1304" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1305">
@@ -35665,7 +35665,7 @@
         <v>3</v>
       </c>
       <c r="G1305" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1306">
@@ -35692,7 +35692,7 @@
         <v>3</v>
       </c>
       <c r="G1306" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1307">
@@ -35719,7 +35719,7 @@
         <v>3</v>
       </c>
       <c r="G1307" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1308">
@@ -35746,7 +35746,7 @@
         <v>3</v>
       </c>
       <c r="G1308" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1309">
@@ -35773,7 +35773,7 @@
         <v>3</v>
       </c>
       <c r="G1309" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1310">
@@ -35800,7 +35800,7 @@
         <v>3</v>
       </c>
       <c r="G1310" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1311">
@@ -35827,7 +35827,7 @@
         <v>3</v>
       </c>
       <c r="G1311" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1312">
@@ -35854,7 +35854,7 @@
         <v>3</v>
       </c>
       <c r="G1312" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1313">
@@ -35881,7 +35881,7 @@
         <v>3</v>
       </c>
       <c r="G1313" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1314">
@@ -35908,7 +35908,7 @@
         <v>3</v>
       </c>
       <c r="G1314" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1315">
@@ -35935,7 +35935,7 @@
         <v>3</v>
       </c>
       <c r="G1315" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1316">
@@ -35962,7 +35962,7 @@
         <v>3</v>
       </c>
       <c r="G1316" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1317">
@@ -35989,7 +35989,7 @@
         <v>3</v>
       </c>
       <c r="G1317" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1318">
@@ -36016,7 +36016,7 @@
         <v>3</v>
       </c>
       <c r="G1318" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1319">
@@ -36043,7 +36043,7 @@
         <v>3</v>
       </c>
       <c r="G1319" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1320">
@@ -36070,7 +36070,7 @@
         <v>3</v>
       </c>
       <c r="G1320" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
     <row r="1321">
@@ -36097,7 +36097,7 @@
         <v>3</v>
       </c>
       <c r="G1321" s="2" t="n">
-        <v>46197.95051278598</v>
+        <v>46198.42723569326</v>
       </c>
     </row>
   </sheetData>

</xml_diff>